<commit_message>
feat(inventory): add read-only mode and improve excel export
- Implement read-only mode for inventory movement based on user permissions
- Enhance Excel template exporter to support dynamic header mapping
- Add support for named ranges in Excel export functionality
</commit_message>
<xml_diff>
--- a/src/Spherical/wwwroot/plantillas/MovimientoInventario.xlsx
+++ b/src/Spherical/wwwroot/plantillas/MovimientoInventario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Proyectos\Spherikal\Spherical\src\Spherical\wwwroot\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D6A110-6228-4200-A87C-FE51980D1888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981768DA-7740-4690-A1F0-69A849BF7964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-10870" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -259,78 +259,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -339,13 +320,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -631,456 +624,257 @@
   <dimension ref="B1:N33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="3.77734375" style="1" customWidth="1"/>
-    <col min="4" max="12" width="8.77734375" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="3.109375" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="3.77734375" customWidth="1"/>
+    <col min="4" max="12" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="24" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="25"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
     </row>
     <row r="3" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="6"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="8"/>
+      <c r="B3" s="2"/>
+      <c r="L3" s="3"/>
     </row>
     <row r="4" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="20" t="s">
+      <c r="C4" s="27"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="37"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="21"/>
-      <c r="L4" s="22"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="28"/>
     </row>
     <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="6"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="8"/>
+      <c r="B5" s="2"/>
+      <c r="L5" s="3"/>
     </row>
     <row r="6" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="5"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="25"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="12"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="8"/>
+      <c r="B7" s="35"/>
+      <c r="L7" s="3"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="12"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="8"/>
+      <c r="B8" s="35"/>
+      <c r="L8" s="3"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B9" s="12"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="8"/>
+      <c r="B9" s="35"/>
+      <c r="L9" s="3"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="12"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="8"/>
+      <c r="B10" s="35"/>
+      <c r="L10" s="3"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="12"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="8"/>
+      <c r="B11" s="35"/>
+      <c r="L11" s="3"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="12"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="8"/>
+      <c r="B12" s="35"/>
+      <c r="L12" s="3"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="12"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="8"/>
+      <c r="B13" s="35"/>
+      <c r="L13" s="3"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="12"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="8"/>
+      <c r="B14" s="35"/>
+      <c r="L14" s="3"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="12"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="8"/>
+      <c r="B15" s="35"/>
+      <c r="L15" s="3"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B16" s="12"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="8"/>
+      <c r="B16" s="35"/>
+      <c r="L16" s="3"/>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B17" s="12"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="8"/>
+      <c r="B17" s="35"/>
+      <c r="L17" s="3"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B18" s="12"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="8"/>
+      <c r="B18" s="35"/>
+      <c r="L18" s="3"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B19" s="12"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-      <c r="L19" s="8"/>
+      <c r="B19" s="35"/>
+      <c r="L19" s="3"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B20" s="12"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="8"/>
+      <c r="B20" s="35"/>
+      <c r="L20" s="3"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B21" s="12"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="8"/>
+      <c r="B21" s="35"/>
+      <c r="L21" s="3"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B22" s="12"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="8"/>
+      <c r="B22" s="35"/>
+      <c r="L22" s="3"/>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B23" s="12"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="8"/>
+      <c r="B23" s="35"/>
+      <c r="L23" s="3"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B24" s="12"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="8"/>
+      <c r="B24" s="35"/>
+      <c r="L24" s="3"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B25" s="12"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="8"/>
+      <c r="B25" s="35"/>
+      <c r="L25" s="3"/>
     </row>
     <row r="26" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="13"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="11"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="6"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B27" s="35" t="s">
+      <c r="B27" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="36"/>
-      <c r="K27" s="36"/>
-      <c r="L27" s="37"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="19"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B28" s="32"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="34"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="31"/>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B29" s="38"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="39"/>
-      <c r="J29" s="39"/>
-      <c r="K29" s="39"/>
-      <c r="L29" s="40"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="31"/>
     </row>
     <row r="30" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="41"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="42"/>
-      <c r="J30" s="42"/>
-      <c r="K30" s="42"/>
-      <c r="L30" s="43"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="34"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="27" t="s">
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="29"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
+      <c r="L31" s="14"/>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B32" s="6"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
-      <c r="L32" s="8"/>
+      <c r="B32" s="2"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="2"/>
+      <c r="L32" s="3"/>
     </row>
     <row r="33" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="9"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="10"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
-      <c r="L33" s="11"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B28:L28"/>
+  <mergeCells count="7">
+    <mergeCell ref="B28:L30"/>
     <mergeCell ref="B27:L27"/>
-    <mergeCell ref="B29:L29"/>
-    <mergeCell ref="B30:L30"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="C6:L6"/>
     <mergeCell ref="B4:C4"/>

</xml_diff>